<commit_message>
Fall back to "EINSTEIN Albert, Al" format for coding student names
</commit_message>
<xml_diff>
--- a/example_files/1ma1df01/empty_for_notes.xlsx
+++ b/example_files/1ma1df01/empty_for_notes.xlsx
@@ -34,16 +34,16 @@
     <t>Student</t>
   </si>
   <si>
-    <t>albert.enstn</t>
-  </si>
-  <si>
-    <t>gabriel.crmr</t>
-  </si>
-  <si>
-    <t>marie.cr</t>
-  </si>
-  <si>
-    <t>richard.fynmn</t>
+    <t>EINSTEIN Albert</t>
+  </si>
+  <si>
+    <t>CRAMER Gabriel</t>
+  </si>
+  <si>
+    <t>CURIE Marie</t>
+  </si>
+  <si>
+    <t>FEYNMANN Richard</t>
   </si>
   <si>
     <t>Total</t>
@@ -130,7 +130,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -565,8 +565,9 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G6:G9">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
-      <formula>4</formula>
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="between">
+      <formula>-100.0</formula>
+      <formula>3.945</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>